<commit_message>
Redesign economic indicators sheet with time-series columns
Sheet 2 now split into Monthly and Quarterly sections.
Each row shows 6 consecutive periods (oldest→newest) as columns
rather than a single latest/prior comparison. Within each
frequency section, indicators are grouped by topic (Inflation,
Labour, Monetary Policy, etc.).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013rcLoLZUmUtk85cDansF3e
</commit_message>
<xml_diff>
--- a/market_dashboard_20260620.xlsx
+++ b/market_dashboard_20260620.xlsx
@@ -648,17 +648,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -669,50 +669,8 @@
       </c>
     </row>
     <row r="2" ht="5" customHeight="1"/>
-    <row r="3" ht="34" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Indicator</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Freq</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Latest Value</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Latest Date</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Prior Value</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Prior Date</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Change</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Trend ▲▼</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="60" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+    <row r="3" ht="60" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>FRED API key required for economic data.
 Get a free key at: fred.stlouisfed.org/docs/api/api_key.html
@@ -720,11 +678,11 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5"/>
-    <row r="6"/>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A4:H6"/>
+    <mergeCell ref="A3:H5"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>